<commit_message>
chore: update agrivision test reports
</commit_message>
<xml_diff>
--- a/agrivision-tests/reports/Appium_Report.xlsx
+++ b/agrivision-tests/reports/Appium_Report.xlsx
@@ -442,7 +442,7 @@
         <v>Passed</v>
       </c>
       <c r="G2" t="str">
-        <v>28ms</v>
+        <v>38ms</v>
       </c>
     </row>
     <row r="3">
@@ -465,7 +465,7 @@
         <v>Passed</v>
       </c>
       <c r="G3" t="str">
-        <v>34ms</v>
+        <v>12ms</v>
       </c>
     </row>
     <row r="4">
@@ -488,7 +488,7 @@
         <v>Passed</v>
       </c>
       <c r="G4" t="str">
-        <v>12ms</v>
+        <v>52ms</v>
       </c>
     </row>
     <row r="5">
@@ -534,7 +534,7 @@
         <v>Passed</v>
       </c>
       <c r="G6" t="str">
-        <v>42ms</v>
+        <v>45ms</v>
       </c>
     </row>
     <row r="7">
@@ -557,7 +557,7 @@
         <v>Passed</v>
       </c>
       <c r="G7" t="str">
-        <v>48ms</v>
+        <v>59ms</v>
       </c>
     </row>
     <row r="8">
@@ -580,7 +580,7 @@
         <v>Passed</v>
       </c>
       <c r="G8" t="str">
-        <v>16ms</v>
+        <v>50ms</v>
       </c>
     </row>
     <row r="9">
@@ -603,7 +603,7 @@
         <v>Passed</v>
       </c>
       <c r="G9" t="str">
-        <v>33ms</v>
+        <v>22ms</v>
       </c>
     </row>
     <row r="10">
@@ -626,7 +626,7 @@
         <v>Passed</v>
       </c>
       <c r="G10" t="str">
-        <v>41ms</v>
+        <v>29ms</v>
       </c>
     </row>
     <row r="11">
@@ -649,7 +649,7 @@
         <v>Passed</v>
       </c>
       <c r="G11" t="str">
-        <v>58ms</v>
+        <v>15ms</v>
       </c>
     </row>
     <row r="12">
@@ -672,7 +672,7 @@
         <v>Passed</v>
       </c>
       <c r="G12" t="str">
-        <v>39ms</v>
+        <v>52ms</v>
       </c>
     </row>
     <row r="13">
@@ -695,7 +695,7 @@
         <v>Passed</v>
       </c>
       <c r="G13" t="str">
-        <v>18ms</v>
+        <v>22ms</v>
       </c>
     </row>
     <row r="14">
@@ -718,7 +718,7 @@
         <v>Passed</v>
       </c>
       <c r="G14" t="str">
-        <v>58ms</v>
+        <v>40ms</v>
       </c>
     </row>
     <row r="15">
@@ -741,7 +741,7 @@
         <v>Passed</v>
       </c>
       <c r="G15" t="str">
-        <v>18ms</v>
+        <v>37ms</v>
       </c>
     </row>
     <row r="16">
@@ -764,7 +764,7 @@
         <v>Passed</v>
       </c>
       <c r="G16" t="str">
-        <v>20ms</v>
+        <v>15ms</v>
       </c>
     </row>
     <row r="17">
@@ -787,7 +787,7 @@
         <v>Passed</v>
       </c>
       <c r="G17" t="str">
-        <v>15ms</v>
+        <v>58ms</v>
       </c>
     </row>
     <row r="18">
@@ -810,7 +810,7 @@
         <v>Passed</v>
       </c>
       <c r="G18" t="str">
-        <v>46ms</v>
+        <v>16ms</v>
       </c>
     </row>
     <row r="19">
@@ -833,7 +833,7 @@
         <v>Passed</v>
       </c>
       <c r="G19" t="str">
-        <v>53ms</v>
+        <v>24ms</v>
       </c>
     </row>
     <row r="20">
@@ -856,7 +856,7 @@
         <v>Passed</v>
       </c>
       <c r="G20" t="str">
-        <v>41ms</v>
+        <v>54ms</v>
       </c>
     </row>
     <row r="21">
@@ -879,7 +879,7 @@
         <v>Passed</v>
       </c>
       <c r="G21" t="str">
-        <v>52ms</v>
+        <v>27ms</v>
       </c>
     </row>
     <row r="22">
@@ -902,7 +902,7 @@
         <v>Passed</v>
       </c>
       <c r="G22" t="str">
-        <v>56ms</v>
+        <v>52ms</v>
       </c>
     </row>
     <row r="23">
@@ -925,7 +925,7 @@
         <v>Passed</v>
       </c>
       <c r="G23" t="str">
-        <v>40ms</v>
+        <v>39ms</v>
       </c>
     </row>
     <row r="24">
@@ -948,7 +948,7 @@
         <v>Passed</v>
       </c>
       <c r="G24" t="str">
-        <v>16ms</v>
+        <v>10ms</v>
       </c>
     </row>
     <row r="25">
@@ -971,7 +971,7 @@
         <v>Passed</v>
       </c>
       <c r="G25" t="str">
-        <v>15ms</v>
+        <v>27ms</v>
       </c>
     </row>
     <row r="26">
@@ -994,7 +994,7 @@
         <v>Passed</v>
       </c>
       <c r="G26" t="str">
-        <v>31ms</v>
+        <v>56ms</v>
       </c>
     </row>
     <row r="27">
@@ -1017,7 +1017,7 @@
         <v>Passed</v>
       </c>
       <c r="G27" t="str">
-        <v>32ms</v>
+        <v>11ms</v>
       </c>
     </row>
     <row r="28">
@@ -1040,7 +1040,7 @@
         <v>Passed</v>
       </c>
       <c r="G28" t="str">
-        <v>24ms</v>
+        <v>56ms</v>
       </c>
     </row>
     <row r="29">
@@ -1063,7 +1063,7 @@
         <v>Passed</v>
       </c>
       <c r="G29" t="str">
-        <v>33ms</v>
+        <v>16ms</v>
       </c>
     </row>
     <row r="30">
@@ -1086,7 +1086,7 @@
         <v>Passed</v>
       </c>
       <c r="G30" t="str">
-        <v>40ms</v>
+        <v>18ms</v>
       </c>
     </row>
     <row r="31">
@@ -1109,7 +1109,7 @@
         <v>Passed</v>
       </c>
       <c r="G31" t="str">
-        <v>30ms</v>
+        <v>20ms</v>
       </c>
     </row>
     <row r="32">
@@ -1132,7 +1132,7 @@
         <v>Passed</v>
       </c>
       <c r="G32" t="str">
-        <v>58ms</v>
+        <v>22ms</v>
       </c>
     </row>
     <row r="33">
@@ -1155,7 +1155,7 @@
         <v>Passed</v>
       </c>
       <c r="G33" t="str">
-        <v>26ms</v>
+        <v>17ms</v>
       </c>
     </row>
     <row r="34">
@@ -1178,7 +1178,7 @@
         <v>Passed</v>
       </c>
       <c r="G34" t="str">
-        <v>15ms</v>
+        <v>57ms</v>
       </c>
     </row>
     <row r="35">
@@ -1201,7 +1201,7 @@
         <v>Passed</v>
       </c>
       <c r="G35" t="str">
-        <v>53ms</v>
+        <v>59ms</v>
       </c>
     </row>
     <row r="36">
@@ -1224,7 +1224,7 @@
         <v>Passed</v>
       </c>
       <c r="G36" t="str">
-        <v>16ms</v>
+        <v>38ms</v>
       </c>
     </row>
     <row r="37">
@@ -1247,7 +1247,7 @@
         <v>Passed</v>
       </c>
       <c r="G37" t="str">
-        <v>15ms</v>
+        <v>30ms</v>
       </c>
     </row>
     <row r="38">
@@ -1270,7 +1270,7 @@
         <v>Passed</v>
       </c>
       <c r="G38" t="str">
-        <v>11ms</v>
+        <v>46ms</v>
       </c>
     </row>
     <row r="39">
@@ -1293,7 +1293,7 @@
         <v>Passed</v>
       </c>
       <c r="G39" t="str">
-        <v>33ms</v>
+        <v>45ms</v>
       </c>
     </row>
     <row r="40">
@@ -1316,7 +1316,7 @@
         <v>Passed</v>
       </c>
       <c r="G40" t="str">
-        <v>31ms</v>
+        <v>44ms</v>
       </c>
     </row>
     <row r="41">
@@ -1339,7 +1339,7 @@
         <v>Passed</v>
       </c>
       <c r="G41" t="str">
-        <v>13ms</v>
+        <v>22ms</v>
       </c>
     </row>
     <row r="42">
@@ -1362,7 +1362,7 @@
         <v>Passed</v>
       </c>
       <c r="G42" t="str">
-        <v>10ms</v>
+        <v>59ms</v>
       </c>
     </row>
     <row r="43">
@@ -1385,7 +1385,7 @@
         <v>Passed</v>
       </c>
       <c r="G43" t="str">
-        <v>47ms</v>
+        <v>33ms</v>
       </c>
     </row>
     <row r="44">
@@ -1408,7 +1408,7 @@
         <v>Passed</v>
       </c>
       <c r="G44" t="str">
-        <v>32ms</v>
+        <v>28ms</v>
       </c>
     </row>
     <row r="45">
@@ -1431,7 +1431,7 @@
         <v>Passed</v>
       </c>
       <c r="G45" t="str">
-        <v>55ms</v>
+        <v>53ms</v>
       </c>
     </row>
     <row r="46">
@@ -1454,7 +1454,7 @@
         <v>Passed</v>
       </c>
       <c r="G46" t="str">
-        <v>36ms</v>
+        <v>25ms</v>
       </c>
     </row>
     <row r="47">
@@ -1477,7 +1477,7 @@
         <v>Passed</v>
       </c>
       <c r="G47" t="str">
-        <v>54ms</v>
+        <v>43ms</v>
       </c>
     </row>
     <row r="48">
@@ -1500,7 +1500,7 @@
         <v>Passed</v>
       </c>
       <c r="G48" t="str">
-        <v>31ms</v>
+        <v>11ms</v>
       </c>
     </row>
     <row r="49">
@@ -1523,7 +1523,7 @@
         <v>Passed</v>
       </c>
       <c r="G49" t="str">
-        <v>37ms</v>
+        <v>19ms</v>
       </c>
     </row>
     <row r="50">
@@ -1546,7 +1546,7 @@
         <v>Passed</v>
       </c>
       <c r="G50" t="str">
-        <v>49ms</v>
+        <v>41ms</v>
       </c>
     </row>
     <row r="51">
@@ -1569,7 +1569,7 @@
         <v>Passed</v>
       </c>
       <c r="G51" t="str">
-        <v>50ms</v>
+        <v>24ms</v>
       </c>
     </row>
     <row r="52">
@@ -1592,7 +1592,7 @@
         <v>Passed</v>
       </c>
       <c r="G52" t="str">
-        <v>40ms</v>
+        <v>50ms</v>
       </c>
     </row>
     <row r="53">
@@ -1615,7 +1615,7 @@
         <v>Passed</v>
       </c>
       <c r="G53" t="str">
-        <v>42ms</v>
+        <v>36ms</v>
       </c>
     </row>
     <row r="54">
@@ -1638,7 +1638,7 @@
         <v>Passed</v>
       </c>
       <c r="G54" t="str">
-        <v>54ms</v>
+        <v>13ms</v>
       </c>
     </row>
     <row r="55">
@@ -1661,7 +1661,7 @@
         <v>Passed</v>
       </c>
       <c r="G55" t="str">
-        <v>54ms</v>
+        <v>33ms</v>
       </c>
     </row>
     <row r="56">
@@ -1684,7 +1684,7 @@
         <v>Passed</v>
       </c>
       <c r="G56" t="str">
-        <v>48ms</v>
+        <v>38ms</v>
       </c>
     </row>
     <row r="57">
@@ -1707,7 +1707,7 @@
         <v>Passed</v>
       </c>
       <c r="G57" t="str">
-        <v>10ms</v>
+        <v>51ms</v>
       </c>
     </row>
     <row r="58">
@@ -1730,7 +1730,7 @@
         <v>Passed</v>
       </c>
       <c r="G58" t="str">
-        <v>45ms</v>
+        <v>10ms</v>
       </c>
     </row>
     <row r="59">
@@ -1753,7 +1753,7 @@
         <v>Passed</v>
       </c>
       <c r="G59" t="str">
-        <v>31ms</v>
+        <v>33ms</v>
       </c>
     </row>
     <row r="60">
@@ -1776,7 +1776,7 @@
         <v>Passed</v>
       </c>
       <c r="G60" t="str">
-        <v>27ms</v>
+        <v>10ms</v>
       </c>
     </row>
     <row r="61">
@@ -1799,7 +1799,7 @@
         <v>Passed</v>
       </c>
       <c r="G61" t="str">
-        <v>33ms</v>
+        <v>50ms</v>
       </c>
     </row>
     <row r="62">
@@ -1822,7 +1822,7 @@
         <v>Passed</v>
       </c>
       <c r="G62" t="str">
-        <v>26ms</v>
+        <v>23ms</v>
       </c>
     </row>
     <row r="63">
@@ -1845,7 +1845,7 @@
         <v>Passed</v>
       </c>
       <c r="G63" t="str">
-        <v>16ms</v>
+        <v>43ms</v>
       </c>
     </row>
     <row r="64">
@@ -1868,7 +1868,7 @@
         <v>Passed</v>
       </c>
       <c r="G64" t="str">
-        <v>14ms</v>
+        <v>30ms</v>
       </c>
     </row>
     <row r="65">
@@ -1891,7 +1891,7 @@
         <v>Passed</v>
       </c>
       <c r="G65" t="str">
-        <v>44ms</v>
+        <v>54ms</v>
       </c>
     </row>
     <row r="66">
@@ -1914,7 +1914,7 @@
         <v>Passed</v>
       </c>
       <c r="G66" t="str">
-        <v>47ms</v>
+        <v>57ms</v>
       </c>
     </row>
     <row r="67">
@@ -1937,7 +1937,7 @@
         <v>Passed</v>
       </c>
       <c r="G67" t="str">
-        <v>37ms</v>
+        <v>54ms</v>
       </c>
     </row>
     <row r="68">
@@ -1960,7 +1960,7 @@
         <v>Passed</v>
       </c>
       <c r="G68" t="str">
-        <v>43ms</v>
+        <v>10ms</v>
       </c>
     </row>
     <row r="69">
@@ -1983,7 +1983,7 @@
         <v>Passed</v>
       </c>
       <c r="G69" t="str">
-        <v>35ms</v>
+        <v>55ms</v>
       </c>
     </row>
     <row r="70">
@@ -2006,7 +2006,7 @@
         <v>Passed</v>
       </c>
       <c r="G70" t="str">
-        <v>12ms</v>
+        <v>19ms</v>
       </c>
     </row>
     <row r="71">
@@ -2029,7 +2029,7 @@
         <v>Passed</v>
       </c>
       <c r="G71" t="str">
-        <v>36ms</v>
+        <v>58ms</v>
       </c>
     </row>
     <row r="72">
@@ -2052,7 +2052,7 @@
         <v>Passed</v>
       </c>
       <c r="G72" t="str">
-        <v>55ms</v>
+        <v>52ms</v>
       </c>
     </row>
     <row r="73">
@@ -2075,7 +2075,7 @@
         <v>Passed</v>
       </c>
       <c r="G73" t="str">
-        <v>50ms</v>
+        <v>40ms</v>
       </c>
     </row>
     <row r="74">
@@ -2098,7 +2098,7 @@
         <v>Passed</v>
       </c>
       <c r="G74" t="str">
-        <v>54ms</v>
+        <v>57ms</v>
       </c>
     </row>
     <row r="75">
@@ -2121,7 +2121,7 @@
         <v>Passed</v>
       </c>
       <c r="G75" t="str">
-        <v>32ms</v>
+        <v>31ms</v>
       </c>
     </row>
     <row r="76">
@@ -2144,7 +2144,7 @@
         <v>Passed</v>
       </c>
       <c r="G76" t="str">
-        <v>14ms</v>
+        <v>23ms</v>
       </c>
     </row>
     <row r="77">
@@ -2167,7 +2167,7 @@
         <v>Passed</v>
       </c>
       <c r="G77" t="str">
-        <v>20ms</v>
+        <v>40ms</v>
       </c>
     </row>
     <row r="78">
@@ -2190,7 +2190,7 @@
         <v>Passed</v>
       </c>
       <c r="G78" t="str">
-        <v>18ms</v>
+        <v>22ms</v>
       </c>
     </row>
     <row r="79">
@@ -2213,7 +2213,7 @@
         <v>Passed</v>
       </c>
       <c r="G79" t="str">
-        <v>13ms</v>
+        <v>24ms</v>
       </c>
     </row>
     <row r="80">
@@ -2236,7 +2236,7 @@
         <v>Passed</v>
       </c>
       <c r="G80" t="str">
-        <v>49ms</v>
+        <v>58ms</v>
       </c>
     </row>
     <row r="81">
@@ -2259,7 +2259,7 @@
         <v>Passed</v>
       </c>
       <c r="G81" t="str">
-        <v>23ms</v>
+        <v>37ms</v>
       </c>
     </row>
     <row r="82">
@@ -2282,7 +2282,7 @@
         <v>Passed</v>
       </c>
       <c r="G82" t="str">
-        <v>37ms</v>
+        <v>22ms</v>
       </c>
     </row>
     <row r="83">
@@ -2305,7 +2305,7 @@
         <v>Passed</v>
       </c>
       <c r="G83" t="str">
-        <v>26ms</v>
+        <v>57ms</v>
       </c>
     </row>
     <row r="84">
@@ -2328,7 +2328,7 @@
         <v>Passed</v>
       </c>
       <c r="G84" t="str">
-        <v>32ms</v>
+        <v>42ms</v>
       </c>
     </row>
     <row r="85">
@@ -2374,7 +2374,7 @@
         <v>Passed</v>
       </c>
       <c r="G86" t="str">
-        <v>49ms</v>
+        <v>11ms</v>
       </c>
     </row>
     <row r="87">
@@ -2397,7 +2397,7 @@
         <v>Passed</v>
       </c>
       <c r="G87" t="str">
-        <v>20ms</v>
+        <v>55ms</v>
       </c>
     </row>
     <row r="88">
@@ -2420,7 +2420,7 @@
         <v>Passed</v>
       </c>
       <c r="G88" t="str">
-        <v>23ms</v>
+        <v>51ms</v>
       </c>
     </row>
     <row r="89">
@@ -2443,7 +2443,7 @@
         <v>Passed</v>
       </c>
       <c r="G89" t="str">
-        <v>54ms</v>
+        <v>46ms</v>
       </c>
     </row>
     <row r="90">
@@ -2466,7 +2466,7 @@
         <v>Passed</v>
       </c>
       <c r="G90" t="str">
-        <v>45ms</v>
+        <v>54ms</v>
       </c>
     </row>
     <row r="91">
@@ -2489,7 +2489,7 @@
         <v>Passed</v>
       </c>
       <c r="G91" t="str">
-        <v>22ms</v>
+        <v>27ms</v>
       </c>
     </row>
     <row r="92">
@@ -2512,7 +2512,7 @@
         <v>Passed</v>
       </c>
       <c r="G92" t="str">
-        <v>51ms</v>
+        <v>53ms</v>
       </c>
     </row>
     <row r="93">
@@ -2535,7 +2535,7 @@
         <v>Passed</v>
       </c>
       <c r="G93" t="str">
-        <v>24ms</v>
+        <v>17ms</v>
       </c>
     </row>
     <row r="94">
@@ -2558,7 +2558,7 @@
         <v>Passed</v>
       </c>
       <c r="G94" t="str">
-        <v>53ms</v>
+        <v>17ms</v>
       </c>
     </row>
     <row r="95">
@@ -2581,7 +2581,7 @@
         <v>Passed</v>
       </c>
       <c r="G95" t="str">
-        <v>41ms</v>
+        <v>46ms</v>
       </c>
     </row>
     <row r="96">
@@ -2604,7 +2604,7 @@
         <v>Passed</v>
       </c>
       <c r="G96" t="str">
-        <v>15ms</v>
+        <v>43ms</v>
       </c>
     </row>
     <row r="97">
@@ -2627,7 +2627,7 @@
         <v>Passed</v>
       </c>
       <c r="G97" t="str">
-        <v>37ms</v>
+        <v>33ms</v>
       </c>
     </row>
     <row r="98">
@@ -2650,7 +2650,7 @@
         <v>Passed</v>
       </c>
       <c r="G98" t="str">
-        <v>55ms</v>
+        <v>22ms</v>
       </c>
     </row>
     <row r="99">
@@ -2673,7 +2673,7 @@
         <v>Passed</v>
       </c>
       <c r="G99" t="str">
-        <v>24ms</v>
+        <v>47ms</v>
       </c>
     </row>
     <row r="100">
@@ -2696,7 +2696,7 @@
         <v>Passed</v>
       </c>
       <c r="G100" t="str">
-        <v>22ms</v>
+        <v>21ms</v>
       </c>
     </row>
     <row r="101">
@@ -2719,7 +2719,7 @@
         <v>Passed</v>
       </c>
       <c r="G101" t="str">
-        <v>50ms</v>
+        <v>39ms</v>
       </c>
     </row>
     <row r="102">
@@ -2742,7 +2742,7 @@
         <v>Passed</v>
       </c>
       <c r="G102" t="str">
-        <v>48ms</v>
+        <v>52ms</v>
       </c>
     </row>
     <row r="103">
@@ -2765,7 +2765,7 @@
         <v>Passed</v>
       </c>
       <c r="G103" t="str">
-        <v>14ms</v>
+        <v>26ms</v>
       </c>
     </row>
     <row r="104">
@@ -2788,7 +2788,7 @@
         <v>Passed</v>
       </c>
       <c r="G104" t="str">
-        <v>25ms</v>
+        <v>59ms</v>
       </c>
     </row>
     <row r="105">
@@ -2811,7 +2811,7 @@
         <v>Passed</v>
       </c>
       <c r="G105" t="str">
-        <v>17ms</v>
+        <v>16ms</v>
       </c>
     </row>
     <row r="106">
@@ -2834,7 +2834,7 @@
         <v>Passed</v>
       </c>
       <c r="G106" t="str">
-        <v>37ms</v>
+        <v>23ms</v>
       </c>
     </row>
     <row r="107">
@@ -2857,7 +2857,7 @@
         <v>Passed</v>
       </c>
       <c r="G107" t="str">
-        <v>47ms</v>
+        <v>40ms</v>
       </c>
     </row>
     <row r="108">
@@ -2880,7 +2880,7 @@
         <v>Passed</v>
       </c>
       <c r="G108" t="str">
-        <v>25ms</v>
+        <v>52ms</v>
       </c>
     </row>
     <row r="109">
@@ -2903,7 +2903,7 @@
         <v>Passed</v>
       </c>
       <c r="G109" t="str">
-        <v>29ms</v>
+        <v>28ms</v>
       </c>
     </row>
     <row r="110">
@@ -2926,7 +2926,7 @@
         <v>Passed</v>
       </c>
       <c r="G110" t="str">
-        <v>40ms</v>
+        <v>12ms</v>
       </c>
     </row>
     <row r="111">
@@ -2949,7 +2949,7 @@
         <v>Passed</v>
       </c>
       <c r="G111" t="str">
-        <v>15ms</v>
+        <v>23ms</v>
       </c>
     </row>
     <row r="112">
@@ -2972,7 +2972,7 @@
         <v>Passed</v>
       </c>
       <c r="G112" t="str">
-        <v>19ms</v>
+        <v>48ms</v>
       </c>
     </row>
     <row r="113">
@@ -2995,7 +2995,7 @@
         <v>Passed</v>
       </c>
       <c r="G113" t="str">
-        <v>27ms</v>
+        <v>47ms</v>
       </c>
     </row>
     <row r="114">
@@ -3018,7 +3018,7 @@
         <v>Passed</v>
       </c>
       <c r="G114" t="str">
-        <v>16ms</v>
+        <v>44ms</v>
       </c>
     </row>
     <row r="115">
@@ -3041,7 +3041,7 @@
         <v>Passed</v>
       </c>
       <c r="G115" t="str">
-        <v>16ms</v>
+        <v>31ms</v>
       </c>
     </row>
     <row r="116">
@@ -3064,7 +3064,7 @@
         <v>Passed</v>
       </c>
       <c r="G116" t="str">
-        <v>43ms</v>
+        <v>20ms</v>
       </c>
     </row>
     <row r="117">
@@ -3087,7 +3087,7 @@
         <v>Passed</v>
       </c>
       <c r="G117" t="str">
-        <v>15ms</v>
+        <v>52ms</v>
       </c>
     </row>
     <row r="118">
@@ -3110,7 +3110,7 @@
         <v>Passed</v>
       </c>
       <c r="G118" t="str">
-        <v>17ms</v>
+        <v>12ms</v>
       </c>
     </row>
     <row r="119">
@@ -3133,7 +3133,7 @@
         <v>Passed</v>
       </c>
       <c r="G119" t="str">
-        <v>29ms</v>
+        <v>34ms</v>
       </c>
     </row>
     <row r="120">
@@ -3156,7 +3156,7 @@
         <v>Passed</v>
       </c>
       <c r="G120" t="str">
-        <v>48ms</v>
+        <v>51ms</v>
       </c>
     </row>
     <row r="121">
@@ -3179,7 +3179,7 @@
         <v>Passed</v>
       </c>
       <c r="G121" t="str">
-        <v>45ms</v>
+        <v>40ms</v>
       </c>
     </row>
     <row r="122">
@@ -3202,7 +3202,7 @@
         <v>Passed</v>
       </c>
       <c r="G122" t="str">
-        <v>51ms</v>
+        <v>55ms</v>
       </c>
     </row>
     <row r="123">
@@ -3225,7 +3225,7 @@
         <v>Passed</v>
       </c>
       <c r="G123" t="str">
-        <v>20ms</v>
+        <v>37ms</v>
       </c>
     </row>
     <row r="124">
@@ -3248,7 +3248,7 @@
         <v>Passed</v>
       </c>
       <c r="G124" t="str">
-        <v>49ms</v>
+        <v>38ms</v>
       </c>
     </row>
     <row r="125">
@@ -3271,7 +3271,7 @@
         <v>Passed</v>
       </c>
       <c r="G125" t="str">
-        <v>21ms</v>
+        <v>58ms</v>
       </c>
     </row>
     <row r="126">
@@ -3294,7 +3294,7 @@
         <v>Passed</v>
       </c>
       <c r="G126" t="str">
-        <v>25ms</v>
+        <v>47ms</v>
       </c>
     </row>
     <row r="127">
@@ -3317,7 +3317,7 @@
         <v>Passed</v>
       </c>
       <c r="G127" t="str">
-        <v>47ms</v>
+        <v>14ms</v>
       </c>
     </row>
     <row r="128">
@@ -3340,7 +3340,7 @@
         <v>Passed</v>
       </c>
       <c r="G128" t="str">
-        <v>10ms</v>
+        <v>37ms</v>
       </c>
     </row>
     <row r="129">
@@ -3363,7 +3363,7 @@
         <v>Passed</v>
       </c>
       <c r="G129" t="str">
-        <v>12ms</v>
+        <v>44ms</v>
       </c>
     </row>
     <row r="130">
@@ -3386,7 +3386,7 @@
         <v>Passed</v>
       </c>
       <c r="G130" t="str">
-        <v>22ms</v>
+        <v>40ms</v>
       </c>
     </row>
     <row r="131">
@@ -3409,7 +3409,7 @@
         <v>Passed</v>
       </c>
       <c r="G131" t="str">
-        <v>28ms</v>
+        <v>34ms</v>
       </c>
     </row>
     <row r="132">
@@ -3432,7 +3432,7 @@
         <v>Passed</v>
       </c>
       <c r="G132" t="str">
-        <v>14ms</v>
+        <v>35ms</v>
       </c>
     </row>
     <row r="133">
@@ -3478,7 +3478,7 @@
         <v>Passed</v>
       </c>
       <c r="G134" t="str">
-        <v>48ms</v>
+        <v>33ms</v>
       </c>
     </row>
     <row r="135">
@@ -3501,7 +3501,7 @@
         <v>Passed</v>
       </c>
       <c r="G135" t="str">
-        <v>36ms</v>
+        <v>14ms</v>
       </c>
     </row>
     <row r="136">
@@ -3524,7 +3524,7 @@
         <v>Passed</v>
       </c>
       <c r="G136" t="str">
-        <v>10ms</v>
+        <v>37ms</v>
       </c>
     </row>
     <row r="137">
@@ -3547,7 +3547,7 @@
         <v>Passed</v>
       </c>
       <c r="G137" t="str">
-        <v>24ms</v>
+        <v>36ms</v>
       </c>
     </row>
     <row r="138">
@@ -3570,7 +3570,7 @@
         <v>Passed</v>
       </c>
       <c r="G138" t="str">
-        <v>51ms</v>
+        <v>49ms</v>
       </c>
     </row>
     <row r="139">
@@ -3593,7 +3593,7 @@
         <v>Passed</v>
       </c>
       <c r="G139" t="str">
-        <v>49ms</v>
+        <v>45ms</v>
       </c>
     </row>
     <row r="140">
@@ -3616,7 +3616,7 @@
         <v>Passed</v>
       </c>
       <c r="G140" t="str">
-        <v>45ms</v>
+        <v>51ms</v>
       </c>
     </row>
     <row r="141">
@@ -3639,7 +3639,7 @@
         <v>Passed</v>
       </c>
       <c r="G141" t="str">
-        <v>14ms</v>
+        <v>30ms</v>
       </c>
     </row>
     <row r="142">
@@ -3662,7 +3662,7 @@
         <v>Passed</v>
       </c>
       <c r="G142" t="str">
-        <v>40ms</v>
+        <v>43ms</v>
       </c>
     </row>
     <row r="143">
@@ -3685,7 +3685,7 @@
         <v>Passed</v>
       </c>
       <c r="G143" t="str">
-        <v>22ms</v>
+        <v>36ms</v>
       </c>
     </row>
     <row r="144">
@@ -3708,7 +3708,7 @@
         <v>Passed</v>
       </c>
       <c r="G144" t="str">
-        <v>37ms</v>
+        <v>10ms</v>
       </c>
     </row>
     <row r="145">
@@ -3731,7 +3731,7 @@
         <v>Passed</v>
       </c>
       <c r="G145" t="str">
-        <v>20ms</v>
+        <v>45ms</v>
       </c>
     </row>
     <row r="146">
@@ -3777,7 +3777,7 @@
         <v>Passed</v>
       </c>
       <c r="G147" t="str">
-        <v>57ms</v>
+        <v>16ms</v>
       </c>
     </row>
     <row r="148">
@@ -3800,7 +3800,7 @@
         <v>Passed</v>
       </c>
       <c r="G148" t="str">
-        <v>12ms</v>
+        <v>25ms</v>
       </c>
     </row>
     <row r="149">
@@ -3823,7 +3823,7 @@
         <v>Passed</v>
       </c>
       <c r="G149" t="str">
-        <v>13ms</v>
+        <v>40ms</v>
       </c>
     </row>
     <row r="150">
@@ -3846,7 +3846,7 @@
         <v>Passed</v>
       </c>
       <c r="G150" t="str">
-        <v>43ms</v>
+        <v>58ms</v>
       </c>
     </row>
     <row r="151">
@@ -3869,7 +3869,7 @@
         <v>Passed</v>
       </c>
       <c r="G151" t="str">
-        <v>40ms</v>
+        <v>57ms</v>
       </c>
     </row>
     <row r="152">
@@ -3892,7 +3892,7 @@
         <v>Passed</v>
       </c>
       <c r="G152" t="str">
-        <v>56ms</v>
+        <v>42ms</v>
       </c>
     </row>
     <row r="153">
@@ -3915,7 +3915,7 @@
         <v>Passed</v>
       </c>
       <c r="G153" t="str">
-        <v>17ms</v>
+        <v>30ms</v>
       </c>
     </row>
     <row r="154">
@@ -3938,7 +3938,7 @@
         <v>Passed</v>
       </c>
       <c r="G154" t="str">
-        <v>48ms</v>
+        <v>14ms</v>
       </c>
     </row>
     <row r="155">
@@ -3961,7 +3961,7 @@
         <v>Passed</v>
       </c>
       <c r="G155" t="str">
-        <v>58ms</v>
+        <v>50ms</v>
       </c>
     </row>
     <row r="156">
@@ -3984,7 +3984,7 @@
         <v>Passed</v>
       </c>
       <c r="G156" t="str">
-        <v>25ms</v>
+        <v>53ms</v>
       </c>
     </row>
     <row r="157">
@@ -4007,7 +4007,7 @@
         <v>Passed</v>
       </c>
       <c r="G157" t="str">
-        <v>17ms</v>
+        <v>19ms</v>
       </c>
     </row>
     <row r="158">
@@ -4030,7 +4030,7 @@
         <v>Passed</v>
       </c>
       <c r="G158" t="str">
-        <v>55ms</v>
+        <v>31ms</v>
       </c>
     </row>
     <row r="159">
@@ -4053,7 +4053,7 @@
         <v>Passed</v>
       </c>
       <c r="G159" t="str">
-        <v>16ms</v>
+        <v>45ms</v>
       </c>
     </row>
     <row r="160">
@@ -4076,7 +4076,7 @@
         <v>Passed</v>
       </c>
       <c r="G160" t="str">
-        <v>19ms</v>
+        <v>31ms</v>
       </c>
     </row>
     <row r="161">
@@ -4099,7 +4099,7 @@
         <v>Passed</v>
       </c>
       <c r="G161" t="str">
-        <v>23ms</v>
+        <v>21ms</v>
       </c>
     </row>
     <row r="162">
@@ -4122,7 +4122,7 @@
         <v>Passed</v>
       </c>
       <c r="G162" t="str">
-        <v>14ms</v>
+        <v>50ms</v>
       </c>
     </row>
     <row r="163">
@@ -4145,7 +4145,7 @@
         <v>Passed</v>
       </c>
       <c r="G163" t="str">
-        <v>39ms</v>
+        <v>38ms</v>
       </c>
     </row>
     <row r="164">
@@ -4168,7 +4168,7 @@
         <v>Passed</v>
       </c>
       <c r="G164" t="str">
-        <v>29ms</v>
+        <v>13ms</v>
       </c>
     </row>
     <row r="165">
@@ -4191,7 +4191,7 @@
         <v>Passed</v>
       </c>
       <c r="G165" t="str">
-        <v>55ms</v>
+        <v>48ms</v>
       </c>
     </row>
     <row r="166">
@@ -4214,7 +4214,7 @@
         <v>Passed</v>
       </c>
       <c r="G166" t="str">
-        <v>44ms</v>
+        <v>22ms</v>
       </c>
     </row>
     <row r="167">
@@ -4237,7 +4237,7 @@
         <v>Passed</v>
       </c>
       <c r="G167" t="str">
-        <v>37ms</v>
+        <v>30ms</v>
       </c>
     </row>
     <row r="168">
@@ -4260,7 +4260,7 @@
         <v>Passed</v>
       </c>
       <c r="G168" t="str">
-        <v>22ms</v>
+        <v>45ms</v>
       </c>
     </row>
     <row r="169">
@@ -4283,7 +4283,7 @@
         <v>Passed</v>
       </c>
       <c r="G169" t="str">
-        <v>20ms</v>
+        <v>10ms</v>
       </c>
     </row>
     <row r="170">
@@ -4306,7 +4306,7 @@
         <v>Passed</v>
       </c>
       <c r="G170" t="str">
-        <v>49ms</v>
+        <v>31ms</v>
       </c>
     </row>
     <row r="171">
@@ -4329,7 +4329,7 @@
         <v>Passed</v>
       </c>
       <c r="G171" t="str">
-        <v>20ms</v>
+        <v>36ms</v>
       </c>
     </row>
     <row r="172">
@@ -4352,7 +4352,7 @@
         <v>Passed</v>
       </c>
       <c r="G172" t="str">
-        <v>41ms</v>
+        <v>16ms</v>
       </c>
     </row>
     <row r="173">
@@ -4375,7 +4375,7 @@
         <v>Passed</v>
       </c>
       <c r="G173" t="str">
-        <v>22ms</v>
+        <v>39ms</v>
       </c>
     </row>
     <row r="174">
@@ -4398,7 +4398,7 @@
         <v>Passed</v>
       </c>
       <c r="G174" t="str">
-        <v>37ms</v>
+        <v>55ms</v>
       </c>
     </row>
     <row r="175">
@@ -4421,7 +4421,7 @@
         <v>Passed</v>
       </c>
       <c r="G175" t="str">
-        <v>25ms</v>
+        <v>31ms</v>
       </c>
     </row>
     <row r="176">
@@ -4444,7 +4444,7 @@
         <v>Passed</v>
       </c>
       <c r="G176" t="str">
-        <v>24ms</v>
+        <v>10ms</v>
       </c>
     </row>
     <row r="177">
@@ -4467,7 +4467,7 @@
         <v>Passed</v>
       </c>
       <c r="G177" t="str">
-        <v>34ms</v>
+        <v>56ms</v>
       </c>
     </row>
     <row r="178">
@@ -4490,7 +4490,7 @@
         <v>Passed</v>
       </c>
       <c r="G178" t="str">
-        <v>12ms</v>
+        <v>25ms</v>
       </c>
     </row>
     <row r="179">
@@ -4513,7 +4513,7 @@
         <v>Passed</v>
       </c>
       <c r="G179" t="str">
-        <v>46ms</v>
+        <v>48ms</v>
       </c>
     </row>
     <row r="180">
@@ -4536,7 +4536,7 @@
         <v>Passed</v>
       </c>
       <c r="G180" t="str">
-        <v>43ms</v>
+        <v>20ms</v>
       </c>
     </row>
     <row r="181">
@@ -4559,7 +4559,7 @@
         <v>Passed</v>
       </c>
       <c r="G181" t="str">
-        <v>38ms</v>
+        <v>27ms</v>
       </c>
     </row>
     <row r="182">
@@ -4582,7 +4582,7 @@
         <v>Passed</v>
       </c>
       <c r="G182" t="str">
-        <v>27ms</v>
+        <v>50ms</v>
       </c>
     </row>
     <row r="183">
@@ -4605,7 +4605,7 @@
         <v>Passed</v>
       </c>
       <c r="G183" t="str">
-        <v>37ms</v>
+        <v>30ms</v>
       </c>
     </row>
     <row r="184">
@@ -4628,7 +4628,7 @@
         <v>Passed</v>
       </c>
       <c r="G184" t="str">
-        <v>50ms</v>
+        <v>17ms</v>
       </c>
     </row>
     <row r="185">
@@ -4651,7 +4651,7 @@
         <v>Passed</v>
       </c>
       <c r="G185" t="str">
-        <v>41ms</v>
+        <v>58ms</v>
       </c>
     </row>
     <row r="186">
@@ -4674,7 +4674,7 @@
         <v>Passed</v>
       </c>
       <c r="G186" t="str">
-        <v>45ms</v>
+        <v>54ms</v>
       </c>
     </row>
     <row r="187">
@@ -4697,7 +4697,7 @@
         <v>Passed</v>
       </c>
       <c r="G187" t="str">
-        <v>22ms</v>
+        <v>56ms</v>
       </c>
     </row>
     <row r="188">
@@ -4720,7 +4720,7 @@
         <v>Passed</v>
       </c>
       <c r="G188" t="str">
-        <v>47ms</v>
+        <v>34ms</v>
       </c>
     </row>
     <row r="189">
@@ -4743,7 +4743,7 @@
         <v>Passed</v>
       </c>
       <c r="G189" t="str">
-        <v>59ms</v>
+        <v>29ms</v>
       </c>
     </row>
     <row r="190">
@@ -4766,7 +4766,7 @@
         <v>Passed</v>
       </c>
       <c r="G190" t="str">
-        <v>30ms</v>
+        <v>44ms</v>
       </c>
     </row>
     <row r="191">
@@ -4789,7 +4789,7 @@
         <v>Passed</v>
       </c>
       <c r="G191" t="str">
-        <v>40ms</v>
+        <v>38ms</v>
       </c>
     </row>
     <row r="192">
@@ -4812,7 +4812,7 @@
         <v>Passed</v>
       </c>
       <c r="G192" t="str">
-        <v>47ms</v>
+        <v>10ms</v>
       </c>
     </row>
     <row r="193">
@@ -4835,7 +4835,7 @@
         <v>Passed</v>
       </c>
       <c r="G193" t="str">
-        <v>27ms</v>
+        <v>43ms</v>
       </c>
     </row>
     <row r="194">
@@ -4858,7 +4858,7 @@
         <v>Passed</v>
       </c>
       <c r="G194" t="str">
-        <v>43ms</v>
+        <v>58ms</v>
       </c>
     </row>
     <row r="195">
@@ -4881,7 +4881,7 @@
         <v>Passed</v>
       </c>
       <c r="G195" t="str">
-        <v>32ms</v>
+        <v>42ms</v>
       </c>
     </row>
     <row r="196">
@@ -4904,7 +4904,7 @@
         <v>Passed</v>
       </c>
       <c r="G196" t="str">
-        <v>23ms</v>
+        <v>22ms</v>
       </c>
     </row>
     <row r="197">
@@ -4927,7 +4927,7 @@
         <v>Passed</v>
       </c>
       <c r="G197" t="str">
-        <v>24ms</v>
+        <v>25ms</v>
       </c>
     </row>
     <row r="198">
@@ -4950,7 +4950,7 @@
         <v>Passed</v>
       </c>
       <c r="G198" t="str">
-        <v>16ms</v>
+        <v>13ms</v>
       </c>
     </row>
     <row r="199">
@@ -4973,7 +4973,7 @@
         <v>Passed</v>
       </c>
       <c r="G199" t="str">
-        <v>33ms</v>
+        <v>31ms</v>
       </c>
     </row>
     <row r="200">
@@ -5019,7 +5019,7 @@
         <v>Passed</v>
       </c>
       <c r="G201" t="str">
-        <v>53ms</v>
+        <v>50ms</v>
       </c>
     </row>
     <row r="202">
@@ -5042,7 +5042,7 @@
         <v>Passed</v>
       </c>
       <c r="G202" t="str">
-        <v>11ms</v>
+        <v>14ms</v>
       </c>
     </row>
     <row r="203">
@@ -5065,7 +5065,7 @@
         <v>Passed</v>
       </c>
       <c r="G203" t="str">
-        <v>23ms</v>
+        <v>15ms</v>
       </c>
     </row>
     <row r="204">
@@ -5088,7 +5088,7 @@
         <v>Passed</v>
       </c>
       <c r="G204" t="str">
-        <v>49ms</v>
+        <v>57ms</v>
       </c>
     </row>
     <row r="205">
@@ -5111,7 +5111,7 @@
         <v>Passed</v>
       </c>
       <c r="G205" t="str">
-        <v>17ms</v>
+        <v>29ms</v>
       </c>
     </row>
     <row r="206">
@@ -5134,7 +5134,7 @@
         <v>Passed</v>
       </c>
       <c r="G206" t="str">
-        <v>41ms</v>
+        <v>43ms</v>
       </c>
     </row>
     <row r="207">
@@ -5157,7 +5157,7 @@
         <v>Passed</v>
       </c>
       <c r="G207" t="str">
-        <v>15ms</v>
+        <v>28ms</v>
       </c>
     </row>
     <row r="208">
@@ -5180,7 +5180,7 @@
         <v>Passed</v>
       </c>
       <c r="G208" t="str">
-        <v>23ms</v>
+        <v>40ms</v>
       </c>
     </row>
     <row r="209">
@@ -5203,7 +5203,7 @@
         <v>Passed</v>
       </c>
       <c r="G209" t="str">
-        <v>41ms</v>
+        <v>40ms</v>
       </c>
     </row>
     <row r="210">
@@ -5226,7 +5226,7 @@
         <v>Passed</v>
       </c>
       <c r="G210" t="str">
-        <v>12ms</v>
+        <v>38ms</v>
       </c>
     </row>
     <row r="211">
@@ -5249,7 +5249,7 @@
         <v>Passed</v>
       </c>
       <c r="G211" t="str">
-        <v>59ms</v>
+        <v>26ms</v>
       </c>
     </row>
     <row r="212">
@@ -5272,7 +5272,7 @@
         <v>Passed</v>
       </c>
       <c r="G212" t="str">
-        <v>48ms</v>
+        <v>30ms</v>
       </c>
     </row>
     <row r="213">
@@ -5295,7 +5295,7 @@
         <v>Passed</v>
       </c>
       <c r="G213" t="str">
-        <v>34ms</v>
+        <v>37ms</v>
       </c>
     </row>
     <row r="214">
@@ -5318,7 +5318,7 @@
         <v>Passed</v>
       </c>
       <c r="G214" t="str">
-        <v>33ms</v>
+        <v>25ms</v>
       </c>
     </row>
     <row r="215">
@@ -5341,7 +5341,7 @@
         <v>Passed</v>
       </c>
       <c r="G215" t="str">
-        <v>41ms</v>
+        <v>14ms</v>
       </c>
     </row>
     <row r="216">
@@ -5364,7 +5364,7 @@
         <v>Passed</v>
       </c>
       <c r="G216" t="str">
-        <v>35ms</v>
+        <v>26ms</v>
       </c>
     </row>
     <row r="217">
@@ -5387,7 +5387,7 @@
         <v>Passed</v>
       </c>
       <c r="G217" t="str">
-        <v>28ms</v>
+        <v>37ms</v>
       </c>
     </row>
     <row r="218">
@@ -5410,7 +5410,7 @@
         <v>Passed</v>
       </c>
       <c r="G218" t="str">
-        <v>27ms</v>
+        <v>19ms</v>
       </c>
     </row>
     <row r="219">
@@ -5433,7 +5433,7 @@
         <v>Passed</v>
       </c>
       <c r="G219" t="str">
-        <v>36ms</v>
+        <v>34ms</v>
       </c>
     </row>
     <row r="220">
@@ -5456,7 +5456,7 @@
         <v>Passed</v>
       </c>
       <c r="G220" t="str">
-        <v>39ms</v>
+        <v>29ms</v>
       </c>
     </row>
     <row r="221">
@@ -5479,7 +5479,7 @@
         <v>Passed</v>
       </c>
       <c r="G221" t="str">
-        <v>25ms</v>
+        <v>40ms</v>
       </c>
     </row>
     <row r="222">
@@ -5502,7 +5502,7 @@
         <v>Passed</v>
       </c>
       <c r="G222" t="str">
-        <v>27ms</v>
+        <v>55ms</v>
       </c>
     </row>
     <row r="223">
@@ -5525,7 +5525,7 @@
         <v>Passed</v>
       </c>
       <c r="G223" t="str">
-        <v>35ms</v>
+        <v>18ms</v>
       </c>
     </row>
     <row r="224">
@@ -5548,7 +5548,7 @@
         <v>Passed</v>
       </c>
       <c r="G224" t="str">
-        <v>25ms</v>
+        <v>16ms</v>
       </c>
     </row>
     <row r="225">
@@ -5571,7 +5571,7 @@
         <v>Passed</v>
       </c>
       <c r="G225" t="str">
-        <v>19ms</v>
+        <v>37ms</v>
       </c>
     </row>
     <row r="226">
@@ -5594,7 +5594,7 @@
         <v>Passed</v>
       </c>
       <c r="G226" t="str">
-        <v>14ms</v>
+        <v>57ms</v>
       </c>
     </row>
     <row r="227">
@@ -5617,7 +5617,7 @@
         <v>Passed</v>
       </c>
       <c r="G227" t="str">
-        <v>13ms</v>
+        <v>25ms</v>
       </c>
     </row>
     <row r="228">
@@ -5640,7 +5640,7 @@
         <v>Passed</v>
       </c>
       <c r="G228" t="str">
-        <v>21ms</v>
+        <v>20ms</v>
       </c>
     </row>
     <row r="229">
@@ -5663,7 +5663,7 @@
         <v>Passed</v>
       </c>
       <c r="G229" t="str">
-        <v>16ms</v>
+        <v>38ms</v>
       </c>
     </row>
     <row r="230">
@@ -5686,7 +5686,7 @@
         <v>Passed</v>
       </c>
       <c r="G230" t="str">
-        <v>25ms</v>
+        <v>33ms</v>
       </c>
     </row>
     <row r="231">
@@ -5709,7 +5709,7 @@
         <v>Passed</v>
       </c>
       <c r="G231" t="str">
-        <v>14ms</v>
+        <v>11ms</v>
       </c>
     </row>
     <row r="232">
@@ -5732,7 +5732,7 @@
         <v>Passed</v>
       </c>
       <c r="G232" t="str">
-        <v>12ms</v>
+        <v>56ms</v>
       </c>
     </row>
     <row r="233">
@@ -5755,7 +5755,7 @@
         <v>Passed</v>
       </c>
       <c r="G233" t="str">
-        <v>43ms</v>
+        <v>36ms</v>
       </c>
     </row>
     <row r="234">
@@ -5778,7 +5778,7 @@
         <v>Passed</v>
       </c>
       <c r="G234" t="str">
-        <v>42ms</v>
+        <v>58ms</v>
       </c>
     </row>
     <row r="235">
@@ -5801,7 +5801,7 @@
         <v>Passed</v>
       </c>
       <c r="G235" t="str">
-        <v>49ms</v>
+        <v>22ms</v>
       </c>
     </row>
     <row r="236">
@@ -5824,7 +5824,7 @@
         <v>Passed</v>
       </c>
       <c r="G236" t="str">
-        <v>47ms</v>
+        <v>30ms</v>
       </c>
     </row>
     <row r="237">
@@ -5847,7 +5847,7 @@
         <v>Passed</v>
       </c>
       <c r="G237" t="str">
-        <v>10ms</v>
+        <v>26ms</v>
       </c>
     </row>
     <row r="238">
@@ -5893,7 +5893,7 @@
         <v>Passed</v>
       </c>
       <c r="G239" t="str">
-        <v>33ms</v>
+        <v>15ms</v>
       </c>
     </row>
     <row r="240">
@@ -5916,7 +5916,7 @@
         <v>Passed</v>
       </c>
       <c r="G240" t="str">
-        <v>54ms</v>
+        <v>31ms</v>
       </c>
     </row>
     <row r="241">
@@ -5939,7 +5939,7 @@
         <v>Passed</v>
       </c>
       <c r="G241" t="str">
-        <v>56ms</v>
+        <v>31ms</v>
       </c>
     </row>
     <row r="242">
@@ -5962,7 +5962,7 @@
         <v>Passed</v>
       </c>
       <c r="G242" t="str">
-        <v>16ms</v>
+        <v>54ms</v>
       </c>
     </row>
     <row r="243">
@@ -5985,7 +5985,7 @@
         <v>Passed</v>
       </c>
       <c r="G243" t="str">
-        <v>15ms</v>
+        <v>31ms</v>
       </c>
     </row>
     <row r="244">
@@ -6008,7 +6008,7 @@
         <v>Passed</v>
       </c>
       <c r="G244" t="str">
-        <v>38ms</v>
+        <v>29ms</v>
       </c>
     </row>
     <row r="245">
@@ -6031,7 +6031,7 @@
         <v>Passed</v>
       </c>
       <c r="G245" t="str">
-        <v>12ms</v>
+        <v>20ms</v>
       </c>
     </row>
     <row r="246">
@@ -6054,7 +6054,7 @@
         <v>Passed</v>
       </c>
       <c r="G246" t="str">
-        <v>57ms</v>
+        <v>51ms</v>
       </c>
     </row>
     <row r="247">
@@ -6077,7 +6077,7 @@
         <v>Passed</v>
       </c>
       <c r="G247" t="str">
-        <v>11ms</v>
+        <v>19ms</v>
       </c>
     </row>
     <row r="248">
@@ -6100,7 +6100,7 @@
         <v>Passed</v>
       </c>
       <c r="G248" t="str">
-        <v>36ms</v>
+        <v>50ms</v>
       </c>
     </row>
     <row r="249">
@@ -6123,7 +6123,7 @@
         <v>Passed</v>
       </c>
       <c r="G249" t="str">
-        <v>27ms</v>
+        <v>39ms</v>
       </c>
     </row>
     <row r="250">
@@ -6146,7 +6146,7 @@
         <v>Passed</v>
       </c>
       <c r="G250" t="str">
-        <v>52ms</v>
+        <v>28ms</v>
       </c>
     </row>
     <row r="251">
@@ -6169,7 +6169,7 @@
         <v>Passed</v>
       </c>
       <c r="G251" t="str">
-        <v>52ms</v>
+        <v>33ms</v>
       </c>
     </row>
     <row r="252">
@@ -6192,7 +6192,7 @@
         <v>Passed</v>
       </c>
       <c r="G252" t="str">
-        <v>19ms</v>
+        <v>32ms</v>
       </c>
     </row>
     <row r="253">
@@ -6215,7 +6215,7 @@
         <v>Passed</v>
       </c>
       <c r="G253" t="str">
-        <v>54ms</v>
+        <v>47ms</v>
       </c>
     </row>
     <row r="254">
@@ -6238,7 +6238,7 @@
         <v>Passed</v>
       </c>
       <c r="G254" t="str">
-        <v>38ms</v>
+        <v>46ms</v>
       </c>
     </row>
     <row r="255">
@@ -6261,7 +6261,7 @@
         <v>Passed</v>
       </c>
       <c r="G255" t="str">
-        <v>45ms</v>
+        <v>41ms</v>
       </c>
     </row>
     <row r="256">
@@ -6284,7 +6284,7 @@
         <v>Passed</v>
       </c>
       <c r="G256" t="str">
-        <v>33ms</v>
+        <v>58ms</v>
       </c>
     </row>
     <row r="257">
@@ -6307,7 +6307,7 @@
         <v>Passed</v>
       </c>
       <c r="G257" t="str">
-        <v>31ms</v>
+        <v>50ms</v>
       </c>
     </row>
     <row r="258">
@@ -6330,7 +6330,7 @@
         <v>Passed</v>
       </c>
       <c r="G258" t="str">
-        <v>46ms</v>
+        <v>23ms</v>
       </c>
     </row>
     <row r="259">
@@ -6353,7 +6353,7 @@
         <v>Passed</v>
       </c>
       <c r="G259" t="str">
-        <v>46ms</v>
+        <v>12ms</v>
       </c>
     </row>
     <row r="260">
@@ -6376,7 +6376,7 @@
         <v>Passed</v>
       </c>
       <c r="G260" t="str">
-        <v>48ms</v>
+        <v>53ms</v>
       </c>
     </row>
     <row r="261">
@@ -6399,7 +6399,7 @@
         <v>Passed</v>
       </c>
       <c r="G261" t="str">
-        <v>30ms</v>
+        <v>12ms</v>
       </c>
     </row>
     <row r="262">
@@ -6422,7 +6422,7 @@
         <v>Passed</v>
       </c>
       <c r="G262" t="str">
-        <v>37ms</v>
+        <v>35ms</v>
       </c>
     </row>
     <row r="263">
@@ -6445,7 +6445,7 @@
         <v>Passed</v>
       </c>
       <c r="G263" t="str">
-        <v>22ms</v>
+        <v>49ms</v>
       </c>
     </row>
     <row r="264">
@@ -6468,7 +6468,7 @@
         <v>Passed</v>
       </c>
       <c r="G264" t="str">
-        <v>31ms</v>
+        <v>40ms</v>
       </c>
     </row>
     <row r="265">
@@ -6491,7 +6491,7 @@
         <v>Passed</v>
       </c>
       <c r="G265" t="str">
-        <v>26ms</v>
+        <v>58ms</v>
       </c>
     </row>
     <row r="266">
@@ -6514,7 +6514,7 @@
         <v>Passed</v>
       </c>
       <c r="G266" t="str">
-        <v>15ms</v>
+        <v>39ms</v>
       </c>
     </row>
     <row r="267">
@@ -6537,7 +6537,7 @@
         <v>Passed</v>
       </c>
       <c r="G267" t="str">
-        <v>55ms</v>
+        <v>34ms</v>
       </c>
     </row>
     <row r="268">
@@ -6560,7 +6560,7 @@
         <v>Passed</v>
       </c>
       <c r="G268" t="str">
-        <v>51ms</v>
+        <v>38ms</v>
       </c>
     </row>
     <row r="269">
@@ -6583,7 +6583,7 @@
         <v>Passed</v>
       </c>
       <c r="G269" t="str">
-        <v>10ms</v>
+        <v>14ms</v>
       </c>
     </row>
     <row r="270">
@@ -6629,7 +6629,7 @@
         <v>Passed</v>
       </c>
       <c r="G271" t="str">
-        <v>13ms</v>
+        <v>12ms</v>
       </c>
     </row>
     <row r="272">
@@ -6652,7 +6652,7 @@
         <v>Passed</v>
       </c>
       <c r="G272" t="str">
-        <v>44ms</v>
+        <v>31ms</v>
       </c>
     </row>
     <row r="273">
@@ -6675,7 +6675,7 @@
         <v>Passed</v>
       </c>
       <c r="G273" t="str">
-        <v>40ms</v>
+        <v>35ms</v>
       </c>
     </row>
     <row r="274">
@@ -6698,7 +6698,7 @@
         <v>Passed</v>
       </c>
       <c r="G274" t="str">
-        <v>27ms</v>
+        <v>45ms</v>
       </c>
     </row>
     <row r="275">
@@ -6721,7 +6721,7 @@
         <v>Passed</v>
       </c>
       <c r="G275" t="str">
-        <v>23ms</v>
+        <v>52ms</v>
       </c>
     </row>
     <row r="276">
@@ -6744,7 +6744,7 @@
         <v>Passed</v>
       </c>
       <c r="G276" t="str">
-        <v>47ms</v>
+        <v>29ms</v>
       </c>
     </row>
     <row r="277">
@@ -6767,7 +6767,7 @@
         <v>Passed</v>
       </c>
       <c r="G277" t="str">
-        <v>14ms</v>
+        <v>52ms</v>
       </c>
     </row>
     <row r="278">
@@ -6790,7 +6790,7 @@
         <v>Passed</v>
       </c>
       <c r="G278" t="str">
-        <v>31ms</v>
+        <v>28ms</v>
       </c>
     </row>
     <row r="279">
@@ -6813,7 +6813,7 @@
         <v>Passed</v>
       </c>
       <c r="G279" t="str">
-        <v>14ms</v>
+        <v>34ms</v>
       </c>
     </row>
     <row r="280">
@@ -6836,7 +6836,7 @@
         <v>Passed</v>
       </c>
       <c r="G280" t="str">
-        <v>57ms</v>
+        <v>59ms</v>
       </c>
     </row>
     <row r="281">
@@ -6859,7 +6859,7 @@
         <v>Passed</v>
       </c>
       <c r="G281" t="str">
-        <v>57ms</v>
+        <v>28ms</v>
       </c>
     </row>
     <row r="282">
@@ -6882,7 +6882,7 @@
         <v>Passed</v>
       </c>
       <c r="G282" t="str">
-        <v>26ms</v>
+        <v>49ms</v>
       </c>
     </row>
     <row r="283">
@@ -6905,7 +6905,7 @@
         <v>Passed</v>
       </c>
       <c r="G283" t="str">
-        <v>12ms</v>
+        <v>35ms</v>
       </c>
     </row>
     <row r="284">
@@ -6928,7 +6928,7 @@
         <v>Passed</v>
       </c>
       <c r="G284" t="str">
-        <v>32ms</v>
+        <v>41ms</v>
       </c>
     </row>
     <row r="285">
@@ -6951,7 +6951,7 @@
         <v>Passed</v>
       </c>
       <c r="G285" t="str">
-        <v>53ms</v>
+        <v>28ms</v>
       </c>
     </row>
     <row r="286">
@@ -6974,7 +6974,7 @@
         <v>Passed</v>
       </c>
       <c r="G286" t="str">
-        <v>35ms</v>
+        <v>24ms</v>
       </c>
     </row>
     <row r="287">
@@ -6997,7 +6997,7 @@
         <v>Passed</v>
       </c>
       <c r="G287" t="str">
-        <v>20ms</v>
+        <v>28ms</v>
       </c>
     </row>
     <row r="288">
@@ -7020,7 +7020,7 @@
         <v>Passed</v>
       </c>
       <c r="G288" t="str">
-        <v>38ms</v>
+        <v>57ms</v>
       </c>
     </row>
     <row r="289">
@@ -7043,7 +7043,7 @@
         <v>Passed</v>
       </c>
       <c r="G289" t="str">
-        <v>22ms</v>
+        <v>19ms</v>
       </c>
     </row>
     <row r="290">
@@ -7066,7 +7066,7 @@
         <v>Passed</v>
       </c>
       <c r="G290" t="str">
-        <v>18ms</v>
+        <v>46ms</v>
       </c>
     </row>
     <row r="291">
@@ -7089,7 +7089,7 @@
         <v>Passed</v>
       </c>
       <c r="G291" t="str">
-        <v>19ms</v>
+        <v>41ms</v>
       </c>
     </row>
     <row r="292">
@@ -7112,7 +7112,7 @@
         <v>Failed</v>
       </c>
       <c r="G292" t="str">
-        <v>35ms</v>
+        <v>41ms</v>
       </c>
     </row>
     <row r="293">

</xml_diff>